<commit_message>
drop concentration from the WELAS was being calculated incorrectly
</commit_message>
<xml_diff>
--- a/analysis/warm_activation_data_and_modelling.xlsx
+++ b/analysis/warm_activation_data_and_modelling.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mccikpc2/The University of Manchester Dropbox/Paul Connolly/projects/iSKYLAB01/analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A20DA02-5FAE-5C4F-8F8C-1AA42CBE5FE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23CC916E-22E8-4D4D-85D1-1723C48D23E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4740" yWindow="760" windowWidth="29820" windowHeight="21580" xr2:uid="{8FF09716-CAC9-1442-85DA-6DCA1581684A}"/>
   </bookViews>
@@ -447,14 +447,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
@@ -960,317 +959,307 @@
       <c r="A2" s="4">
         <v>6</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2">
         <v>14</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2">
         <v>20</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2">
         <v>9</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E2" s="5">
         <v>0.77360755933585501</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2">
         <v>0.61</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2">
         <v>1.28</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" t="s">
         <v>46</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="K2" t="s">
         <v>19</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="L2" t="s">
         <v>47</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="M2" t="s">
         <v>20</v>
       </c>
-      <c r="N2" s="5">
+      <c r="N2">
         <v>2272.55054823</v>
       </c>
-      <c r="O2" s="5">
-        <v>242.68669183</v>
-      </c>
-      <c r="P2" s="7"/>
+      <c r="O2">
+        <v>496.66122705999999</v>
+      </c>
+      <c r="P2" s="6"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="4">
         <v>7</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3">
         <v>18</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3">
         <v>21</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3">
         <v>12</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="5">
         <v>0.67855760130550102</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3">
         <v>0.61</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3">
         <v>1.28</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" t="s">
         <v>48</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" t="s">
         <v>22</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="K3" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="L3" t="s">
         <v>49</v>
       </c>
-      <c r="M3" s="5" t="s">
+      <c r="M3" t="s">
         <v>24</v>
       </c>
-      <c r="N3" s="5">
+      <c r="N3">
         <v>2458.9618684000002</v>
       </c>
-      <c r="O3" s="5">
-        <v>379.20164663000003</v>
-      </c>
-      <c r="P3" s="7"/>
+      <c r="O3">
+        <v>776.04072025999994</v>
+      </c>
+      <c r="P3" s="6"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="4">
         <v>8</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4">
         <v>15</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4">
         <v>18</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4">
         <v>10</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="5">
         <v>0.74690748377548999</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4">
         <v>0.61</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4">
         <v>1.28</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" t="s">
         <v>25</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" t="s">
         <v>50</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="J4" t="s">
         <v>26</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="K4" t="s">
         <v>27</v>
       </c>
-      <c r="L4" s="5" t="s">
+      <c r="L4" t="s">
         <v>51</v>
       </c>
-      <c r="M4" s="5" t="s">
+      <c r="M4" t="s">
         <v>28</v>
       </c>
-      <c r="N4" s="5">
+      <c r="N4">
         <v>2564.5208385300002</v>
       </c>
-      <c r="O4" s="5">
-        <v>186.22267500000001</v>
-      </c>
-      <c r="P4" s="7"/>
+      <c r="O4">
+        <v>381.10693906</v>
+      </c>
+      <c r="P4" s="6"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="4">
         <v>9</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5">
         <v>13</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5">
         <v>15</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5">
         <v>9</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="5">
         <v>0.77869596406718899</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5">
         <v>0.61</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5">
         <v>1.28</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" t="s">
         <v>29</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" t="s">
         <v>52</v>
       </c>
-      <c r="J5" s="5" t="s">
+      <c r="J5" t="s">
         <v>30</v>
       </c>
-      <c r="K5" s="5" t="s">
+      <c r="K5" t="s">
         <v>31</v>
       </c>
-      <c r="L5" s="5" t="s">
+      <c r="L5" t="s">
         <v>53</v>
       </c>
-      <c r="M5" s="5" t="s">
+      <c r="M5" t="s">
         <v>32</v>
       </c>
-      <c r="N5" s="5">
+      <c r="N5">
         <v>2693.80518274</v>
       </c>
-      <c r="O5" s="5">
-        <v>206.42190577</v>
-      </c>
-      <c r="P5" s="7"/>
+      <c r="O5">
+        <v>422.44490722</v>
+      </c>
+      <c r="P5" s="6"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" s="4">
         <v>10</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6">
         <v>13</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6">
         <v>15</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6">
         <v>9</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="5">
         <v>0.77477340673249595</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6">
         <v>0.61</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6">
         <v>1.28</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" t="s">
         <v>33</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" t="s">
         <v>54</v>
       </c>
-      <c r="J6" s="5" t="s">
+      <c r="J6" t="s">
         <v>34</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="K6" t="s">
         <v>35</v>
       </c>
-      <c r="L6" s="5" t="s">
+      <c r="L6" t="s">
         <v>55</v>
       </c>
-      <c r="M6" s="5" t="s">
+      <c r="M6" t="s">
         <v>36</v>
       </c>
-      <c r="N6" s="5">
+      <c r="N6">
         <v>2449.4828249100001</v>
       </c>
-      <c r="O6" s="5">
-        <v>230.17777163</v>
-      </c>
-      <c r="P6" s="7"/>
+      <c r="O6">
+        <v>471.06157178000001</v>
+      </c>
+      <c r="P6" s="6"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" s="4">
         <v>11</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7">
         <v>17</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7">
         <v>19</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7">
         <v>11</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="5">
         <v>0.73587286267528496</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7">
         <v>0.61</v>
       </c>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5" t="s">
+      <c r="H7" t="s">
         <v>37</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" t="s">
         <v>56</v>
       </c>
-      <c r="J7" s="5" t="s">
+      <c r="J7" t="s">
         <v>38</v>
       </c>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5">
+      <c r="N7">
         <v>2509.3976526800002</v>
       </c>
-      <c r="O7" s="5">
-        <v>156.13633798000001</v>
-      </c>
-      <c r="P7" s="7"/>
+      <c r="O7">
+        <v>319.53488930999998</v>
+      </c>
+      <c r="P7" s="6"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" s="4">
         <v>12</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8">
         <v>14</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8">
         <v>16</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8">
         <v>10</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="5">
         <v>0.75244681090566401</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8">
         <v>1.28</v>
       </c>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5" t="s">
+      <c r="H8" t="s">
         <v>39</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" t="s">
         <v>57</v>
       </c>
-      <c r="J8" s="5" t="s">
+      <c r="J8" t="s">
         <v>40</v>
       </c>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="5"/>
-      <c r="O8" s="5"/>
-      <c r="P8" s="7" t="s">
+      <c r="P8" s="6" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1278,245 +1267,223 @@
       <c r="A9" s="4">
         <v>13</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9">
         <v>13</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9">
         <v>15</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9">
         <v>10</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="5">
         <v>0.75268565250988595</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9">
         <v>1.28</v>
       </c>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5" t="s">
+      <c r="H9" t="s">
         <v>41</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="I9" t="s">
         <v>58</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="J9" t="s">
         <v>42</v>
       </c>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5">
+      <c r="N9">
         <v>470.76719104</v>
       </c>
-      <c r="O9" s="5">
-        <v>126.62354567</v>
-      </c>
-      <c r="P9" s="7"/>
+      <c r="O9">
+        <v>259.13660570000002</v>
+      </c>
+      <c r="P9" s="6"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="4">
         <v>14</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10">
         <v>15</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10">
         <v>17</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10">
         <v>9</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="5">
         <v>0.77310396385688296</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10">
         <v>1.28</v>
       </c>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5" t="s">
+      <c r="H10" t="s">
         <v>43</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="I10" t="s">
         <v>59</v>
       </c>
-      <c r="J10" s="5" t="s">
+      <c r="J10" t="s">
         <v>44</v>
       </c>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5">
+      <c r="N10">
         <v>1677.55071374</v>
       </c>
-      <c r="O10" s="5">
-        <v>257.31781970999998</v>
-      </c>
-      <c r="P10" s="7"/>
+      <c r="O10">
+        <v>526.60400585000002</v>
+      </c>
+      <c r="P10" s="6"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" s="4">
         <v>15</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11">
         <v>10.5</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11">
         <v>13</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11">
         <v>9</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="5">
         <v>0.77769949177724496</v>
       </c>
-      <c r="F11" s="5">
+      <c r="F11">
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5" t="s">
+      <c r="H11" t="s">
         <v>45</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I11" t="s">
         <v>60</v>
       </c>
-      <c r="J11" s="5" t="s">
+      <c r="J11" t="s">
         <v>61</v>
       </c>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5">
+      <c r="N11">
         <v>1345.6287211599999</v>
       </c>
-      <c r="O11" s="5">
-        <v>148.99250673</v>
-      </c>
-      <c r="P11" s="7"/>
+      <c r="O11">
+        <v>304.91495293000003</v>
+      </c>
+      <c r="P11" s="6"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" s="4">
         <v>16</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12">
         <v>10.5</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12">
         <v>13</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12">
         <v>9</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="5">
         <v>0.77624010569497603</v>
       </c>
-      <c r="F12" s="5">
+      <c r="F12">
         <v>0.61</v>
       </c>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5" t="s">
+      <c r="H12" t="s">
         <v>62</v>
       </c>
-      <c r="I12" s="5" t="s">
+      <c r="I12" t="s">
         <v>63</v>
       </c>
-      <c r="J12" s="5" t="s">
+      <c r="J12" t="s">
         <v>64</v>
       </c>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5">
+      <c r="N12">
         <v>804.17988771</v>
       </c>
-      <c r="O12" s="5">
-        <v>129.68510769</v>
-      </c>
-      <c r="P12" s="7"/>
+      <c r="O12">
+        <v>265.40212910999998</v>
+      </c>
+      <c r="P12" s="6"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" s="4">
         <v>17</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13">
         <v>1.67</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13">
         <v>2</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13">
         <v>1.25</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="5">
         <v>0.78781301699605499</v>
       </c>
-      <c r="F13" s="5">
+      <c r="F13">
         <v>0.61</v>
       </c>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5" t="s">
+      <c r="H13" t="s">
         <v>65</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="I13" t="s">
         <v>66</v>
       </c>
-      <c r="J13" s="5" t="s">
+      <c r="J13" t="s">
         <v>67</v>
       </c>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5">
+      <c r="N13">
         <v>1703.7358157799999</v>
       </c>
-      <c r="O13" s="5">
-        <v>376.01818028999998</v>
-      </c>
-      <c r="P13" s="7"/>
+      <c r="O13">
+        <v>769.52571818000001</v>
+      </c>
+      <c r="P13" s="6"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" s="4">
         <v>18</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14">
         <v>9</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14">
         <v>11</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14">
         <v>7</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="5">
         <v>0.77611139214627201</v>
       </c>
-      <c r="F14" s="5">
+      <c r="F14">
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="G14" s="5">
+      <c r="G14">
         <v>1.28</v>
       </c>
-      <c r="H14" s="5" t="s">
+      <c r="H14" t="s">
         <v>68</v>
       </c>
-      <c r="I14" s="5" t="s">
+      <c r="I14" t="s">
         <v>69</v>
       </c>
-      <c r="J14" s="5" t="s">
+      <c r="J14" t="s">
         <v>70</v>
       </c>
-      <c r="K14" s="5" t="s">
+      <c r="K14" t="s">
         <v>71</v>
       </c>
-      <c r="L14" s="5" t="s">
+      <c r="L14" t="s">
         <v>72</v>
       </c>
-      <c r="M14" s="5" t="s">
+      <c r="M14" t="s">
         <v>73</v>
       </c>
-      <c r="N14" s="5"/>
-      <c r="O14" s="5"/>
-      <c r="P14" s="7" t="s">
+      <c r="P14" s="6" t="s">
         <v>89</v>
       </c>
     </row>
@@ -1524,89 +1491,89 @@
       <c r="A15" s="4">
         <v>19</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15">
         <v>14</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15">
         <v>16</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15">
         <v>10</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="5">
         <v>0.75248218441166903</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15">
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G15">
         <v>1.28</v>
       </c>
-      <c r="H15" s="5" t="s">
+      <c r="H15" t="s">
         <v>74</v>
       </c>
-      <c r="I15" s="5" t="s">
+      <c r="I15" t="s">
         <v>75</v>
       </c>
-      <c r="J15" s="5" t="s">
+      <c r="J15" t="s">
         <v>76</v>
       </c>
-      <c r="K15" s="5" t="s">
+      <c r="K15" t="s">
         <v>77</v>
       </c>
-      <c r="L15" s="5" t="s">
+      <c r="L15" t="s">
         <v>78</v>
       </c>
-      <c r="M15" s="5" t="s">
+      <c r="M15" t="s">
         <v>79</v>
       </c>
-      <c r="N15" s="5">
+      <c r="N15">
         <v>1719.6167825699999</v>
       </c>
-      <c r="O15" s="5">
-        <v>247.09868076999999</v>
-      </c>
-      <c r="P15" s="7"/>
+      <c r="O15">
+        <v>505.69041537999999</v>
+      </c>
+      <c r="P15" s="6"/>
     </row>
     <row r="16" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="8">
+      <c r="A16" s="7">
         <v>28</v>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="8">
         <v>11</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="8">
         <v>13</v>
       </c>
-      <c r="D16" s="9">
+      <c r="D16" s="8">
         <v>7</v>
       </c>
-      <c r="E16" s="10">
+      <c r="E16" s="9">
         <v>0.84776854359447995</v>
       </c>
-      <c r="F16" s="9">
+      <c r="F16" s="8">
         <v>0.61</v>
       </c>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9" t="s">
+      <c r="G16" s="8"/>
+      <c r="H16" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="I16" s="9" t="s">
+      <c r="I16" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="J16" s="9" t="s">
+      <c r="J16" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="K16" s="9"/>
-      <c r="L16" s="9"/>
-      <c r="M16" s="9"/>
-      <c r="N16" s="9">
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="8"/>
+      <c r="N16" s="8">
         <v>1891.1348361299999</v>
       </c>
-      <c r="O16" s="9">
-        <v>177.04628738</v>
-      </c>
-      <c r="P16" s="11"/>
+      <c r="O16" s="8">
+        <v>358.84343482999998</v>
+      </c>
+      <c r="P16" s="10"/>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">

</xml_diff>